<commit_message>
[Resource Add] 스킬 아이콘 및 Addressables 경로 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -21,19 +21,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <x:si>
-    <x:t>Skill_CrimsonShield_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RottenTomato_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_TomatoFlare_01</x:t>
-  </x:si>
-  <x:si>
     <x:t>Skill_RedHeat_01</x:t>
   </x:si>
   <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
     <x:t>토마토플레어</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍의 보호막</x:t>
   </x:si>
   <x:si>
     <x:t>(name)</x:t>
@@ -42,22 +39,31 @@
     <x:t>붉은 열기</x:t>
   </x:si>
   <x:si>
-    <x:t>선홍의 보호막</x:t>
+    <x:t>string</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
+    <x:t>썩은 토마토</x:t>
   </x:si>
   <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
-    <x:t>썩은 토마토</x:t>
+    <x:t>IconPath</x:t>
   </x:si>
   <x:si>
-    <x:t>Id</x:t>
+    <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
   </x:si>
   <x:si>
     <x:t>뜨겁게 달아오른 화염 토마토를 던져 폭발을 일으킨다.</x:t>
@@ -66,28 +72,22 @@
     <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
   </x:si>
   <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
+    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
   </x:si>
   <x:si>
-    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
+    <x:t>Skill_CrimsonShield_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_TomatoFlare_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RottenTomato_01</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -877,51 +877,51 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
     </x:row>
     <x:row r="2" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B3" s="4" t="s">
+      <x:c r="D3" s="14" t="s">
         <x:v>9</x:v>
-      </x:c>
-      <x:c r="C3" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="s">
-        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A4" s="6" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E4" s="5"/>
       <x:c r="F4" s="5"/>
@@ -937,16 +937,16 @@
     </x:row>
     <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>1</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B5" s="7" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E5" s="5"/>
       <x:c r="F5" s="5"/>
@@ -962,16 +962,16 @@
     </x:row>
     <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A6" s="7" t="s">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>15</x:v>
       </x:c>
       <x:c r="E6" s="5"/>
       <x:c r="F6" s="5"/>
@@ -987,16 +987,16 @@
     </x:row>
     <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5"/>

</xml_diff>

<commit_message>
[Add - Skill Data] PrefabPath 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -19,66 +19,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+  <x:si>
+    <x:t>2DObject/Skill_RedHeat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_CrimsonShield</x:t>
+  </x:si>
   <x:si>
     <x:t>Id</x:t>
   </x:si>
   <x:si>
+    <x:t>Skill_RedHeat_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토</x:t>
+  </x:si>
+  <x:si>
+    <x:t>붉은 열기</x:t>
+  </x:si>
+  <x:si>
     <x:t>토마토플레어</x:t>
   </x:si>
   <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
-    <x:t>썩은 토마토</x:t>
-  </x:si>
-  <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
     <x:t>선홍의 보호막</x:t>
   </x:si>
   <x:si>
-    <x:t>붉은 열기</x:t>
+    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
   </x:si>
   <x:si>
     <x:t>IconPath</x:t>
   </x:si>
   <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
     <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RedHeat_01</x:t>
+    <x:t>PrefabPath</x:t>
   </x:si>
   <x:si>
     <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
   </x:si>
   <x:si>
+    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
+    <x:t>2DObject/Skill_TomatoFlare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_RottenTomato</x:t>
   </x:si>
   <x:si>
     <x:t>Skill_TomatoFlare_01</x:t>
@@ -877,53 +892,61 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
     </x:row>
-    <x:row r="2" spans="1:4" ht="15.75" customHeight="1">
+    <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:4" ht="15.75" customHeight="1">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="4" t="s">
-        <x:v>9</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>8</x:v>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A4" s="6" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="s">
-        <x:v>17</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E4" s="5"/>
+      <x:c r="E4" s="5" t="s">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
@@ -937,18 +960,20 @@
     </x:row>
     <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B5" s="7" t="s">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E5" s="5"/>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E5" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
@@ -962,18 +987,20 @@
     </x:row>
     <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A6" s="7" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E6" s="5"/>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
@@ -987,18 +1014,20 @@
     </x:row>
     <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>18</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E7" s="5"/>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E7" s="5" t="s">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>

</xml_diff>

<commit_message>
[Fix - Skill Data] 스킬 순서 변경
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -21,64 +21,73 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토플레어</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍의 보호막</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토</x:t>
+  </x:si>
+  <x:si>
+    <x:t>붉은 열기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RedHeat_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_CrimsonShield</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
     <x:t>2DObject/Skill_RedHeat</x:t>
   </x:si>
   <x:si>
-    <x:t>2DObject/Skill_CrimsonShield</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RedHeat_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토</x:t>
-  </x:si>
-  <x:si>
-    <x:t>붉은 열기</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토플레어</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍의 보호막</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PrefabPath</x:t>
+    <x:t>Skill_RottenTomato_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_CrimsonShield_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_TomatoFlare_01</x:t>
   </x:si>
   <x:si>
     <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
@@ -94,15 +103,6 @@
   </x:si>
   <x:si>
     <x:t>2DObject/Skill_RottenTomato</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_TomatoFlare_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_CrimsonShield_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RottenTomato_01</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -892,60 +892,60 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
     </x:row>
     <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C3" s="4" t="s">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A4" s="6" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="s">
         <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A4" s="6" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>23</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
@@ -958,21 +958,21 @@
       <x:c r="N4" s="5"/>
       <x:c r="O4" s="5"/>
     </x:row>
-    <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
+    <x:row r="5" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>13</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
@@ -985,21 +985,21 @@
       <x:c r="N5" s="5"/>
       <x:c r="O5" s="5"/>
     </x:row>
-    <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A6" s="7" t="s">
-        <x:v>26</x:v>
+    <x:row r="6" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A6" s="6" t="s">
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
@@ -1012,21 +1012,21 @@
       <x:c r="N6" s="5"/>
       <x:c r="O6" s="5"/>
     </x:row>
-    <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A7" s="6" t="s">
+    <x:row r="7" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A7" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>22</x:v>
+      <x:c r="C7" s="7" t="s">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5"/>
@@ -1039,10 +1039,10 @@
       <x:c r="N7" s="5"/>
       <x:c r="O7" s="5"/>
     </x:row>
-    <x:row r="8" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A8" s="8"/>
-      <x:c r="B8" s="8"/>
-      <x:c r="C8" s="8"/>
+    <x:row r="8" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A8" s="6"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="7"/>
       <x:c r="D8" s="5"/>
       <x:c r="E8" s="5"/>
       <x:c r="F8" s="5"/>
@@ -1056,10 +1056,10 @@
       <x:c r="N8" s="5"/>
       <x:c r="O8" s="5"/>
     </x:row>
-    <x:row r="9" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A9" s="8"/>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8"/>
+    <x:row r="9" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
       <x:c r="D9" s="5"/>
       <x:c r="E9" s="5"/>
       <x:c r="F9" s="5"/>
@@ -1073,10 +1073,10 @@
       <x:c r="N9" s="5"/>
       <x:c r="O9" s="5"/>
     </x:row>
-    <x:row r="10" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A10" s="9"/>
-      <x:c r="B10" s="9"/>
-      <x:c r="C10" s="9"/>
+    <x:row r="10" spans="1:15" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A10" s="6"/>
+      <x:c r="B10" s="6"/>
+      <x:c r="C10" s="6"/>
       <x:c r="D10" s="5"/>
       <x:c r="E10" s="5"/>
       <x:c r="F10" s="5"/>

</xml_diff>

<commit_message>
[Add - Skill Data] MaxUseCount 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -19,42 +19,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+  <x:si>
+    <x:t>MaxUseCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_CrimsonShield_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_TomatoFlare_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_RedHeat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RottenTomato_01</x:t>
+  </x:si>
   <x:si>
     <x:t>Skill_RedHeat_01</x:t>
   </x:si>
   <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_RedHeat</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_CrimsonShield_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RottenTomato_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_TomatoFlare_01</x:t>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
   </x:si>
   <x:si>
+    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>2DObject/Skill_CrimsonShield</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
   </x:si>
   <x:si>
     <x:t>PrefabPath</x:t>
@@ -63,37 +75,31 @@
     <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
+    <x:t>썩은 토마토</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍의 보호막</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토플레어</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
   </x:si>
   <x:si>
     <x:t>붉은 열기</x:t>
   </x:si>
   <x:si>
-    <x:t>썩은 토마토</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍의 보호막</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토플레어</x:t>
+    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
   </x:si>
   <x:si>
     <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
@@ -195,7 +201,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border>
       <x:left>
         <x:color auto="1"/>
@@ -224,22 +230,47 @@
         <x:color rgb="ff000000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="ff000000"/>
+      </x:left>
+      <x:right>
+        <x:color auto="1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="ff000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="ff000000"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color auto="1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color auto="1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color auto="1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color auto="1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <x:alignment horizontal="general" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
@@ -276,8 +307,74 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1">
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -883,406 +980,454 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:O35"/>
+  <x:dimension ref="A1:P35"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="1" width="23" style="3" customWidth="1"/>
-    <x:col min="2" max="2" width="19.5703125" style="3" customWidth="1"/>
-    <x:col min="3" max="3" width="54.109375" style="3" customWidth="1"/>
-    <x:col min="4" max="4" width="27.66796875" style="2" customWidth="1"/>
-    <x:col min="5" max="5" width="30.5703125" style="3" customWidth="1"/>
+    <x:col min="1" max="1" width="23" style="2" customWidth="1"/>
+    <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="54.109375" style="2" customWidth="1"/>
+    <x:col min="4" max="4" width="16.22265625" style="23" customWidth="1"/>
+    <x:col min="5" max="5" width="27.66796875" style="24" customWidth="1"/>
+    <x:col min="6" max="6" width="30.5703125" style="23" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A1" s="4" t="s">
+    <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A1" s="3" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="14"/>
+      <x:c r="D1" s="25"/>
+    </x:row>
+    <x:row r="2" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A2" s="3" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="24" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F2" s="23" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A3" s="4" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D3" s="26" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="34" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F3" s="36" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A4" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D4" s="27">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F4" s="35" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G4" s="5"/>
+      <x:c r="H4" s="5"/>
+      <x:c r="I4" s="5"/>
+      <x:c r="J4" s="5"/>
+      <x:c r="K4" s="5"/>
+      <x:c r="L4" s="5"/>
+      <x:c r="M4" s="5"/>
+      <x:c r="N4" s="5"/>
+      <x:c r="O4" s="5"/>
+      <x:c r="P4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A5" s="6" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D5" s="27">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G5" s="5"/>
+      <x:c r="H5" s="5"/>
+      <x:c r="I5" s="5"/>
+      <x:c r="J5" s="5"/>
+      <x:c r="K5" s="5"/>
+      <x:c r="L5" s="5"/>
+      <x:c r="M5" s="5"/>
+      <x:c r="N5" s="5"/>
+      <x:c r="O5" s="5"/>
+      <x:c r="P5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A6" s="6" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D6" s="28">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="35" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="G6" s="5"/>
+      <x:c r="H6" s="5"/>
+      <x:c r="I6" s="5"/>
+      <x:c r="J6" s="5"/>
+      <x:c r="K6" s="5"/>
+      <x:c r="L6" s="5"/>
+      <x:c r="M6" s="5"/>
+      <x:c r="N6" s="5"/>
+      <x:c r="O6" s="5"/>
+      <x:c r="P6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A7" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D7" s="28">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F7" s="35" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A2" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B2" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C2" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D2" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E2" s="3" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A3" s="5" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D3" s="15" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E3" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A4" s="7" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C4" s="7" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="E4" s="6" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F4" s="6"/>
-      <x:c r="G4" s="6"/>
-      <x:c r="H4" s="6"/>
-      <x:c r="I4" s="6"/>
-      <x:c r="J4" s="6"/>
-      <x:c r="K4" s="6"/>
-      <x:c r="L4" s="6"/>
-      <x:c r="M4" s="6"/>
-      <x:c r="N4" s="6"/>
-      <x:c r="O4" s="6"/>
-    </x:row>
-    <x:row r="5" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A5" s="7" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F5" s="6"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="6"/>
-      <x:c r="I5" s="6"/>
-      <x:c r="J5" s="6"/>
-      <x:c r="K5" s="6"/>
-      <x:c r="L5" s="6"/>
-      <x:c r="M5" s="6"/>
-      <x:c r="N5" s="6"/>
-      <x:c r="O5" s="6"/>
-    </x:row>
-    <x:row r="6" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A6" s="7" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C6" s="8" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F6" s="6"/>
-      <x:c r="G6" s="6"/>
-      <x:c r="H6" s="6"/>
-      <x:c r="I6" s="6"/>
-      <x:c r="J6" s="6"/>
-      <x:c r="K6" s="6"/>
-      <x:c r="L6" s="6"/>
-      <x:c r="M6" s="6"/>
-      <x:c r="N6" s="6"/>
-      <x:c r="O6" s="6"/>
-    </x:row>
-    <x:row r="7" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A7" s="8" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F7" s="6"/>
-      <x:c r="G7" s="6"/>
-      <x:c r="H7" s="6"/>
-      <x:c r="I7" s="6"/>
-      <x:c r="J7" s="6"/>
-      <x:c r="K7" s="6"/>
-      <x:c r="L7" s="6"/>
-      <x:c r="M7" s="6"/>
-      <x:c r="N7" s="6"/>
-      <x:c r="O7" s="6"/>
-    </x:row>
-    <x:row r="8" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="8"/>
-      <x:c r="C8" s="8"/>
-      <x:c r="D8" s="6"/>
-      <x:c r="E8" s="6"/>
-      <x:c r="F8" s="6"/>
-      <x:c r="G8" s="6"/>
-      <x:c r="H8" s="6"/>
-      <x:c r="I8" s="6"/>
-      <x:c r="J8" s="6"/>
-      <x:c r="K8" s="6"/>
-      <x:c r="L8" s="6"/>
-      <x:c r="M8" s="6"/>
-      <x:c r="N8" s="6"/>
-      <x:c r="O8" s="6"/>
-    </x:row>
-    <x:row r="9" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A9" s="8"/>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8"/>
-      <x:c r="D9" s="6"/>
-      <x:c r="E9" s="6"/>
-      <x:c r="F9" s="6"/>
-      <x:c r="G9" s="6"/>
-      <x:c r="H9" s="6"/>
-      <x:c r="I9" s="6"/>
-      <x:c r="J9" s="6"/>
-      <x:c r="K9" s="6"/>
-      <x:c r="L9" s="6"/>
-      <x:c r="M9" s="6"/>
-      <x:c r="N9" s="6"/>
-      <x:c r="O9" s="6"/>
-    </x:row>
-    <x:row r="10" spans="1:15" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A10" s="7"/>
-      <x:c r="B10" s="7"/>
-      <x:c r="C10" s="7"/>
-      <x:c r="D10" s="6"/>
-      <x:c r="E10" s="6"/>
-      <x:c r="F10" s="6"/>
-      <x:c r="G10" s="6"/>
-      <x:c r="H10" s="6"/>
-      <x:c r="I10" s="6"/>
-      <x:c r="J10" s="6"/>
-      <x:c r="K10" s="6"/>
-      <x:c r="L10" s="6"/>
-      <x:c r="M10" s="6"/>
-      <x:c r="N10" s="6"/>
-      <x:c r="O10" s="6"/>
-    </x:row>
-    <x:row r="11" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A11" s="10"/>
-      <x:c r="B11" s="10"/>
-      <x:c r="C11" s="10"/>
-      <x:c r="D11" s="6"/>
-      <x:c r="E11" s="6"/>
-      <x:c r="F11" s="6"/>
-      <x:c r="G11" s="6"/>
-      <x:c r="H11" s="6"/>
-      <x:c r="I11" s="6"/>
-      <x:c r="J11" s="6"/>
-      <x:c r="K11" s="6"/>
-      <x:c r="L11" s="6"/>
-      <x:c r="M11" s="6"/>
-      <x:c r="N11" s="6"/>
-      <x:c r="O11" s="6"/>
-    </x:row>
-    <x:row r="12" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A12" s="9"/>
-      <x:c r="B12" s="9"/>
-      <x:c r="C12" s="9"/>
-      <x:c r="D12" s="6"/>
-      <x:c r="E12" s="6"/>
-      <x:c r="F12" s="6"/>
-      <x:c r="G12" s="6"/>
-      <x:c r="H12" s="6"/>
-      <x:c r="I12" s="6"/>
-      <x:c r="J12" s="6"/>
-      <x:c r="K12" s="6"/>
-      <x:c r="L12" s="6"/>
-      <x:c r="M12" s="6"/>
-      <x:c r="N12" s="6"/>
-      <x:c r="O12" s="6"/>
-    </x:row>
-    <x:row r="13" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A13" s="7"/>
-      <x:c r="B13" s="7"/>
-      <x:c r="C13" s="7"/>
-      <x:c r="D13" s="6"/>
-      <x:c r="E13" s="6"/>
-      <x:c r="F13" s="6"/>
-      <x:c r="G13" s="6"/>
-      <x:c r="H13" s="6"/>
-      <x:c r="I13" s="6"/>
-      <x:c r="J13" s="6"/>
-      <x:c r="K13" s="6"/>
-      <x:c r="L13" s="6"/>
-      <x:c r="M13" s="6"/>
-      <x:c r="N13" s="6"/>
-      <x:c r="O13" s="6"/>
-    </x:row>
-    <x:row r="14" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A14" s="10"/>
-      <x:c r="B14" s="10"/>
-      <x:c r="C14" s="10"/>
-      <x:c r="D14" s="6"/>
-      <x:c r="E14" s="6"/>
-      <x:c r="F14" s="6"/>
-      <x:c r="G14" s="6"/>
-      <x:c r="H14" s="6"/>
-      <x:c r="I14" s="6"/>
-      <x:c r="J14" s="6"/>
-      <x:c r="K14" s="6"/>
-      <x:c r="L14" s="6"/>
-      <x:c r="M14" s="6"/>
-      <x:c r="N14" s="6"/>
-      <x:c r="O14" s="6"/>
-    </x:row>
-    <x:row r="15" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A15" s="10"/>
-      <x:c r="B15" s="10"/>
-      <x:c r="C15" s="10"/>
-      <x:c r="D15" s="6"/>
-      <x:c r="E15" s="6"/>
-      <x:c r="F15" s="6"/>
-      <x:c r="G15" s="6"/>
-      <x:c r="H15" s="6"/>
-      <x:c r="I15" s="6"/>
-      <x:c r="J15" s="6"/>
-      <x:c r="K15" s="6"/>
-      <x:c r="L15" s="6"/>
-      <x:c r="M15" s="6"/>
-      <x:c r="N15" s="6"/>
-      <x:c r="O15" s="6"/>
-    </x:row>
-    <x:row r="16" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A16" s="11"/>
-      <x:c r="B16" s="11"/>
-      <x:c r="C16" s="11"/>
-    </x:row>
-    <x:row r="17" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A17" s="12"/>
-      <x:c r="B17" s="12"/>
-      <x:c r="C17" s="12"/>
-    </x:row>
-    <x:row r="18" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A18" s="12"/>
-      <x:c r="B18" s="12"/>
-      <x:c r="C18" s="12"/>
-    </x:row>
-    <x:row r="19" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A19" s="12"/>
-      <x:c r="B19" s="12"/>
-      <x:c r="C19" s="12"/>
-      <x:c r="D19" s="6"/>
-      <x:c r="E19" s="6"/>
-    </x:row>
-    <x:row r="20" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A20" s="12"/>
-      <x:c r="B20" s="12"/>
-      <x:c r="C20" s="12"/>
-    </x:row>
-    <x:row r="21" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A21" s="12"/>
-      <x:c r="B21" s="12"/>
-      <x:c r="C21" s="12"/>
-    </x:row>
-    <x:row r="22" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A22" s="12"/>
-      <x:c r="B22" s="12"/>
-      <x:c r="C22" s="12"/>
-    </x:row>
-    <x:row r="23" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A23" s="12"/>
-      <x:c r="B23" s="12"/>
-      <x:c r="C23" s="12"/>
-    </x:row>
-    <x:row r="24" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A24" s="12"/>
-      <x:c r="B24" s="12"/>
-      <x:c r="C24" s="12"/>
-    </x:row>
-    <x:row r="25" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A25" s="12"/>
-      <x:c r="B25" s="12"/>
-      <x:c r="C25" s="12"/>
-      <x:c r="E25" s="6"/>
-    </x:row>
-    <x:row r="26" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A26" s="13"/>
-      <x:c r="B26" s="13"/>
-      <x:c r="C26" s="13"/>
-      <x:c r="E26" s="6"/>
-    </x:row>
-    <x:row r="27" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A27" s="13"/>
-      <x:c r="B27" s="13"/>
-      <x:c r="C27" s="13"/>
-      <x:c r="E27" s="6"/>
-    </x:row>
-    <x:row r="28" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A28" s="13"/>
-      <x:c r="B28" s="13"/>
-      <x:c r="C28" s="13"/>
-      <x:c r="E28" s="6"/>
-    </x:row>
-    <x:row r="29" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A29" s="13"/>
-      <x:c r="B29" s="13"/>
-      <x:c r="C29" s="13"/>
-    </x:row>
-    <x:row r="30" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A30" s="13"/>
-      <x:c r="B30" s="13"/>
-      <x:c r="C30" s="13"/>
-    </x:row>
-    <x:row r="31" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A31" s="13"/>
-      <x:c r="B31" s="13"/>
-      <x:c r="C31" s="13"/>
-    </x:row>
-    <x:row r="32" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A32" s="14"/>
-      <x:c r="B32" s="14"/>
-      <x:c r="C32" s="14"/>
-    </x:row>
-    <x:row r="33" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A33" s="14"/>
-      <x:c r="B33" s="14"/>
-      <x:c r="C33" s="14"/>
-    </x:row>
-    <x:row r="34" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A34" s="14"/>
-      <x:c r="B34" s="14"/>
-      <x:c r="C34" s="14"/>
-    </x:row>
-    <x:row r="35" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A35" s="14"/>
-      <x:c r="B35" s="14"/>
-      <x:c r="C35" s="14"/>
+      <x:c r="G7" s="5"/>
+      <x:c r="H7" s="5"/>
+      <x:c r="I7" s="5"/>
+      <x:c r="J7" s="5"/>
+      <x:c r="K7" s="5"/>
+      <x:c r="L7" s="5"/>
+      <x:c r="M7" s="5"/>
+      <x:c r="N7" s="5"/>
+      <x:c r="O7" s="5"/>
+      <x:c r="P7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A8" s="6"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="17"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="35"/>
+      <x:c r="F8" s="35"/>
+      <x:c r="G8" s="5"/>
+      <x:c r="H8" s="5"/>
+      <x:c r="I8" s="5"/>
+      <x:c r="J8" s="5"/>
+      <x:c r="K8" s="5"/>
+      <x:c r="L8" s="5"/>
+      <x:c r="M8" s="5"/>
+      <x:c r="N8" s="5"/>
+      <x:c r="O8" s="5"/>
+      <x:c r="P8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="17"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="35"/>
+      <x:c r="F9" s="35"/>
+      <x:c r="G9" s="5"/>
+      <x:c r="H9" s="5"/>
+      <x:c r="I9" s="5"/>
+      <x:c r="J9" s="5"/>
+      <x:c r="K9" s="5"/>
+      <x:c r="L9" s="5"/>
+      <x:c r="M9" s="5"/>
+      <x:c r="N9" s="5"/>
+      <x:c r="O9" s="5"/>
+      <x:c r="P9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A10" s="6"/>
+      <x:c r="B10" s="6"/>
+      <x:c r="C10" s="16"/>
+      <x:c r="D10" s="27"/>
+      <x:c r="E10" s="35"/>
+      <x:c r="F10" s="35"/>
+      <x:c r="G10" s="5"/>
+      <x:c r="H10" s="5"/>
+      <x:c r="I10" s="5"/>
+      <x:c r="J10" s="5"/>
+      <x:c r="K10" s="5"/>
+      <x:c r="L10" s="5"/>
+      <x:c r="M10" s="5"/>
+      <x:c r="N10" s="5"/>
+      <x:c r="O10" s="5"/>
+      <x:c r="P10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="9"/>
+      <x:c r="C11" s="18"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="35"/>
+      <x:c r="F11" s="35"/>
+      <x:c r="G11" s="5"/>
+      <x:c r="H11" s="5"/>
+      <x:c r="I11" s="5"/>
+      <x:c r="J11" s="5"/>
+      <x:c r="K11" s="5"/>
+      <x:c r="L11" s="5"/>
+      <x:c r="M11" s="5"/>
+      <x:c r="N11" s="5"/>
+      <x:c r="O11" s="5"/>
+      <x:c r="P11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A12" s="8"/>
+      <x:c r="B12" s="8"/>
+      <x:c r="C12" s="19"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="35"/>
+      <x:c r="F12" s="35"/>
+      <x:c r="G12" s="5"/>
+      <x:c r="H12" s="5"/>
+      <x:c r="I12" s="5"/>
+      <x:c r="J12" s="5"/>
+      <x:c r="K12" s="5"/>
+      <x:c r="L12" s="5"/>
+      <x:c r="M12" s="5"/>
+      <x:c r="N12" s="5"/>
+      <x:c r="O12" s="5"/>
+      <x:c r="P12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A13" s="6"/>
+      <x:c r="B13" s="6"/>
+      <x:c r="C13" s="16"/>
+      <x:c r="D13" s="27"/>
+      <x:c r="E13" s="35"/>
+      <x:c r="F13" s="35"/>
+      <x:c r="G13" s="5"/>
+      <x:c r="H13" s="5"/>
+      <x:c r="I13" s="5"/>
+      <x:c r="J13" s="5"/>
+      <x:c r="K13" s="5"/>
+      <x:c r="L13" s="5"/>
+      <x:c r="M13" s="5"/>
+      <x:c r="N13" s="5"/>
+      <x:c r="O13" s="5"/>
+      <x:c r="P13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A14" s="9"/>
+      <x:c r="B14" s="9"/>
+      <x:c r="C14" s="18"/>
+      <x:c r="D14" s="29"/>
+      <x:c r="E14" s="35"/>
+      <x:c r="F14" s="35"/>
+      <x:c r="G14" s="5"/>
+      <x:c r="H14" s="5"/>
+      <x:c r="I14" s="5"/>
+      <x:c r="J14" s="5"/>
+      <x:c r="K14" s="5"/>
+      <x:c r="L14" s="5"/>
+      <x:c r="M14" s="5"/>
+      <x:c r="N14" s="5"/>
+      <x:c r="O14" s="5"/>
+      <x:c r="P14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A15" s="9"/>
+      <x:c r="B15" s="9"/>
+      <x:c r="C15" s="18"/>
+      <x:c r="D15" s="29"/>
+      <x:c r="E15" s="35"/>
+      <x:c r="F15" s="35"/>
+      <x:c r="G15" s="5"/>
+      <x:c r="H15" s="5"/>
+      <x:c r="I15" s="5"/>
+      <x:c r="J15" s="5"/>
+      <x:c r="K15" s="5"/>
+      <x:c r="L15" s="5"/>
+      <x:c r="M15" s="5"/>
+      <x:c r="N15" s="5"/>
+      <x:c r="O15" s="5"/>
+      <x:c r="P15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A16" s="10"/>
+      <x:c r="B16" s="10"/>
+      <x:c r="C16" s="20"/>
+      <x:c r="D16" s="31"/>
+    </x:row>
+    <x:row r="17" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A17" s="11"/>
+      <x:c r="B17" s="11"/>
+      <x:c r="C17" s="20"/>
+      <x:c r="D17" s="31"/>
+    </x:row>
+    <x:row r="18" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A18" s="11"/>
+      <x:c r="B18" s="11"/>
+      <x:c r="C18" s="20"/>
+      <x:c r="D18" s="31"/>
+    </x:row>
+    <x:row r="19" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A19" s="11"/>
+      <x:c r="B19" s="11"/>
+      <x:c r="C19" s="20"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="35"/>
+      <x:c r="F19" s="35"/>
+    </x:row>
+    <x:row r="20" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A20" s="11"/>
+      <x:c r="B20" s="11"/>
+      <x:c r="C20" s="20"/>
+      <x:c r="D20" s="31"/>
+    </x:row>
+    <x:row r="21" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A21" s="11"/>
+      <x:c r="B21" s="11"/>
+      <x:c r="C21" s="20"/>
+      <x:c r="D21" s="31"/>
+    </x:row>
+    <x:row r="22" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A22" s="11"/>
+      <x:c r="B22" s="11"/>
+      <x:c r="C22" s="20"/>
+      <x:c r="D22" s="31"/>
+    </x:row>
+    <x:row r="23" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A23" s="11"/>
+      <x:c r="B23" s="11"/>
+      <x:c r="C23" s="20"/>
+      <x:c r="D23" s="31"/>
+    </x:row>
+    <x:row r="24" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A24" s="11"/>
+      <x:c r="B24" s="11"/>
+      <x:c r="C24" s="20"/>
+      <x:c r="D24" s="31"/>
+    </x:row>
+    <x:row r="25" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A25" s="11"/>
+      <x:c r="B25" s="11"/>
+      <x:c r="C25" s="20"/>
+      <x:c r="D25" s="31"/>
+      <x:c r="F25" s="35"/>
+    </x:row>
+    <x:row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A26" s="12"/>
+      <x:c r="B26" s="12"/>
+      <x:c r="C26" s="21"/>
+      <x:c r="D26" s="32"/>
+      <x:c r="F26" s="35"/>
+    </x:row>
+    <x:row r="27" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A27" s="12"/>
+      <x:c r="B27" s="12"/>
+      <x:c r="C27" s="21"/>
+      <x:c r="D27" s="32"/>
+      <x:c r="F27" s="35"/>
+    </x:row>
+    <x:row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A28" s="12"/>
+      <x:c r="B28" s="12"/>
+      <x:c r="C28" s="21"/>
+      <x:c r="D28" s="32"/>
+      <x:c r="F28" s="35"/>
+    </x:row>
+    <x:row r="29" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A29" s="12"/>
+      <x:c r="B29" s="12"/>
+      <x:c r="C29" s="21"/>
+      <x:c r="D29" s="32"/>
+    </x:row>
+    <x:row r="30" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A30" s="12"/>
+      <x:c r="B30" s="12"/>
+      <x:c r="C30" s="21"/>
+      <x:c r="D30" s="32"/>
+    </x:row>
+    <x:row r="31" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A31" s="12"/>
+      <x:c r="B31" s="12"/>
+      <x:c r="C31" s="21"/>
+      <x:c r="D31" s="32"/>
+    </x:row>
+    <x:row r="32" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A32" s="13"/>
+      <x:c r="B32" s="13"/>
+      <x:c r="C32" s="22"/>
+      <x:c r="D32" s="33"/>
+    </x:row>
+    <x:row r="33" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A33" s="13"/>
+      <x:c r="B33" s="13"/>
+      <x:c r="C33" s="22"/>
+      <x:c r="D33" s="33"/>
+    </x:row>
+    <x:row r="34" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A34" s="13"/>
+      <x:c r="B34" s="13"/>
+      <x:c r="C34" s="22"/>
+      <x:c r="D34" s="33"/>
+    </x:row>
+    <x:row r="35" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A35" s="13"/>
+      <x:c r="B35" s="13"/>
+      <x:c r="C35" s="22"/>
+      <x:c r="D35" s="33"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[Add - Skill Data] RequiredLevel 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -19,96 +19,117 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+  <x:si>
+    <x:t>Icon 경로</x:t>
+  </x:si>
+  <x:si>
+    <x:t>설명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RottenTomato_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_TomatoFlare_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_RedHeat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_CrimsonShield_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RedHeat_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>붉은 열기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍의 보호막</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토마토플레어</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_CrimsonShield</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
   <x:si>
     <x:t>MaxUseCount</x:t>
   </x:si>
   <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_CrimsonShield_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_TomatoFlare_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_RedHeat</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RottenTomato_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RedHeat_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_CrimsonShield</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PrefabPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍의 보호막</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토플레어</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>붉은 열기</x:t>
+    <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_TomatoFlare</x:t>
   </x:si>
   <x:si>
     <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_TomatoFlare</x:t>
-  </x:si>
-  <x:si>
     <x:t>2DObject/Skill_RottenTomato</x:t>
+  </x:si>
+  <x:si>
+    <x:t>사용 가능 횟수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prefab 경로</x:t>
+  </x:si>
+  <x:si>
+    <x:t>요구 레벨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredLevel</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -980,85 +1001,109 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:P35"/>
+  <x:dimension ref="A1:Q35"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="23" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="54.109375" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="16.22265625" style="23" customWidth="1"/>
-    <x:col min="5" max="5" width="27.66796875" style="24" customWidth="1"/>
-    <x:col min="6" max="6" width="30.5703125" style="23" customWidth="1"/>
+    <x:col min="5" max="5" width="18.66796875" style="23" customWidth="1"/>
+    <x:col min="6" max="6" width="27.66796875" style="24" customWidth="1"/>
+    <x:col min="7" max="7" width="30.5703125" style="23" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="14"/>
-      <x:c r="D1" s="25"/>
-    </x:row>
-    <x:row r="2" spans="1:6" ht="15.75" customHeight="1">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C1" s="14" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E1" s="25" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F1" s="24" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G1" s="23" t="s">
+        <x:v>34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C2" s="14" t="s">
-        <x:v>20</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D2" s="25" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" s="24" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F2" s="23" t="s">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6" ht="15.75" customHeight="1">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E2" s="25" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F2" s="24" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G2" s="23" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D3" s="26" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E3" s="26" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F3" s="34" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G3" s="36" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D3" s="26" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="34" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F3" s="36" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="4" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A4" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="6" t="s">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C4" s="16" t="s">
-        <x:v>25</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D4" s="27">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E4" s="35" t="s">
-        <x:v>26</x:v>
+      <x:c r="E4" s="27">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="35" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G4" s="5"/>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="G4" s="35" t="s">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5"/>
       <x:c r="J4" s="5"/>
@@ -1068,27 +1113,30 @@
       <x:c r="N4" s="5"/>
       <x:c r="O4" s="5"/>
       <x:c r="P4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="16" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D5" s="27">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="s">
-        <x:v>12</x:v>
+      <x:c r="E5" s="27">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="35" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="G5" s="5"/>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G5" s="35" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5"/>
       <x:c r="J5" s="5"/>
@@ -1098,27 +1146,30 @@
       <x:c r="N5" s="5"/>
       <x:c r="O5" s="5"/>
       <x:c r="P5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>18</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="17" t="s">
-        <x:v>9</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D6" s="28">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E6" s="35" t="s">
-        <x:v>10</x:v>
+      <x:c r="E6" s="28">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="35" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="G6" s="5"/>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G6" s="35" t="s">
+        <x:v>32</x:v>
+      </x:c>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5"/>
       <x:c r="J6" s="5"/>
@@ -1128,27 +1179,30 @@
       <x:c r="N6" s="5"/>
       <x:c r="O6" s="5"/>
       <x:c r="P6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A7" s="7" t="s">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>21</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>8</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="28">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E7" s="35" t="s">
-        <x:v>11</x:v>
+      <x:c r="E7" s="28">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="35" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="G7" s="5"/>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G7" s="35" t="s">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
@@ -1158,15 +1212,16 @@
       <x:c r="N7" s="5"/>
       <x:c r="O7" s="5"/>
       <x:c r="P7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A8" s="6"/>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="17"/>
       <x:c r="D8" s="28"/>
-      <x:c r="E8" s="35"/>
+      <x:c r="E8" s="28"/>
       <x:c r="F8" s="35"/>
-      <x:c r="G8" s="5"/>
+      <x:c r="G8" s="35"/>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>
@@ -1176,15 +1231,16 @@
       <x:c r="N8" s="5"/>
       <x:c r="O8" s="5"/>
       <x:c r="P8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A9" s="7"/>
       <x:c r="B9" s="7"/>
       <x:c r="C9" s="17"/>
       <x:c r="D9" s="28"/>
-      <x:c r="E9" s="35"/>
+      <x:c r="E9" s="28"/>
       <x:c r="F9" s="35"/>
-      <x:c r="G9" s="5"/>
+      <x:c r="G9" s="35"/>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5"/>
       <x:c r="J9" s="5"/>
@@ -1194,15 +1250,16 @@
       <x:c r="N9" s="5"/>
       <x:c r="O9" s="5"/>
       <x:c r="P9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A10" s="6"/>
       <x:c r="B10" s="6"/>
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="27"/>
-      <x:c r="E10" s="35"/>
+      <x:c r="E10" s="27"/>
       <x:c r="F10" s="35"/>
-      <x:c r="G10" s="5"/>
+      <x:c r="G10" s="35"/>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5"/>
       <x:c r="J10" s="5"/>
@@ -1212,15 +1269,16 @@
       <x:c r="N10" s="5"/>
       <x:c r="O10" s="5"/>
       <x:c r="P10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A11" s="9"/>
       <x:c r="B11" s="9"/>
       <x:c r="C11" s="18"/>
       <x:c r="D11" s="29"/>
-      <x:c r="E11" s="35"/>
+      <x:c r="E11" s="29"/>
       <x:c r="F11" s="35"/>
-      <x:c r="G11" s="5"/>
+      <x:c r="G11" s="35"/>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5"/>
       <x:c r="J11" s="5"/>
@@ -1230,15 +1288,16 @@
       <x:c r="N11" s="5"/>
       <x:c r="O11" s="5"/>
       <x:c r="P11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A12" s="8"/>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="30"/>
-      <x:c r="E12" s="35"/>
+      <x:c r="E12" s="30"/>
       <x:c r="F12" s="35"/>
-      <x:c r="G12" s="5"/>
+      <x:c r="G12" s="35"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5"/>
       <x:c r="J12" s="5"/>
@@ -1248,15 +1307,16 @@
       <x:c r="N12" s="5"/>
       <x:c r="O12" s="5"/>
       <x:c r="P12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A13" s="6"/>
       <x:c r="B13" s="6"/>
       <x:c r="C13" s="16"/>
       <x:c r="D13" s="27"/>
-      <x:c r="E13" s="35"/>
+      <x:c r="E13" s="27"/>
       <x:c r="F13" s="35"/>
-      <x:c r="G13" s="5"/>
+      <x:c r="G13" s="35"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5"/>
       <x:c r="J13" s="5"/>
@@ -1266,15 +1326,16 @@
       <x:c r="N13" s="5"/>
       <x:c r="O13" s="5"/>
       <x:c r="P13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A14" s="9"/>
       <x:c r="B14" s="9"/>
       <x:c r="C14" s="18"/>
       <x:c r="D14" s="29"/>
-      <x:c r="E14" s="35"/>
+      <x:c r="E14" s="29"/>
       <x:c r="F14" s="35"/>
-      <x:c r="G14" s="5"/>
+      <x:c r="G14" s="35"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5"/>
       <x:c r="J14" s="5"/>
@@ -1284,15 +1345,16 @@
       <x:c r="N14" s="5"/>
       <x:c r="O14" s="5"/>
       <x:c r="P14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A15" s="9"/>
       <x:c r="B15" s="9"/>
       <x:c r="C15" s="18"/>
       <x:c r="D15" s="29"/>
-      <x:c r="E15" s="35"/>
+      <x:c r="E15" s="29"/>
       <x:c r="F15" s="35"/>
-      <x:c r="G15" s="5"/>
+      <x:c r="G15" s="35"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5"/>
       <x:c r="J15" s="5"/>
@@ -1302,132 +1364,153 @@
       <x:c r="N15" s="5"/>
       <x:c r="O15" s="5"/>
       <x:c r="P15" s="5"/>
-    </x:row>
-    <x:row r="16" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="Q15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A16" s="10"/>
       <x:c r="B16" s="10"/>
       <x:c r="C16" s="20"/>
       <x:c r="D16" s="31"/>
-    </x:row>
-    <x:row r="17" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E16" s="31"/>
+    </x:row>
+    <x:row r="17" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A17" s="11"/>
       <x:c r="B17" s="11"/>
       <x:c r="C17" s="20"/>
       <x:c r="D17" s="31"/>
-    </x:row>
-    <x:row r="18" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E17" s="31"/>
+    </x:row>
+    <x:row r="18" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A18" s="11"/>
       <x:c r="B18" s="11"/>
       <x:c r="C18" s="20"/>
       <x:c r="D18" s="31"/>
-    </x:row>
-    <x:row r="19" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E18" s="31"/>
+    </x:row>
+    <x:row r="19" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A19" s="11"/>
       <x:c r="B19" s="11"/>
       <x:c r="C19" s="20"/>
       <x:c r="D19" s="31"/>
-      <x:c r="E19" s="35"/>
+      <x:c r="E19" s="31"/>
       <x:c r="F19" s="35"/>
-    </x:row>
-    <x:row r="20" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="G19" s="35"/>
+    </x:row>
+    <x:row r="20" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A20" s="11"/>
       <x:c r="B20" s="11"/>
       <x:c r="C20" s="20"/>
       <x:c r="D20" s="31"/>
-    </x:row>
-    <x:row r="21" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E20" s="31"/>
+    </x:row>
+    <x:row r="21" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A21" s="11"/>
       <x:c r="B21" s="11"/>
       <x:c r="C21" s="20"/>
       <x:c r="D21" s="31"/>
-    </x:row>
-    <x:row r="22" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E21" s="31"/>
+    </x:row>
+    <x:row r="22" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A22" s="11"/>
       <x:c r="B22" s="11"/>
       <x:c r="C22" s="20"/>
       <x:c r="D22" s="31"/>
-    </x:row>
-    <x:row r="23" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E22" s="31"/>
+    </x:row>
+    <x:row r="23" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A23" s="11"/>
       <x:c r="B23" s="11"/>
       <x:c r="C23" s="20"/>
       <x:c r="D23" s="31"/>
-    </x:row>
-    <x:row r="24" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E23" s="31"/>
+    </x:row>
+    <x:row r="24" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A24" s="11"/>
       <x:c r="B24" s="11"/>
       <x:c r="C24" s="20"/>
       <x:c r="D24" s="31"/>
-    </x:row>
-    <x:row r="25" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E24" s="31"/>
+    </x:row>
+    <x:row r="25" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A25" s="11"/>
       <x:c r="B25" s="11"/>
       <x:c r="C25" s="20"/>
       <x:c r="D25" s="31"/>
-      <x:c r="F25" s="35"/>
-    </x:row>
-    <x:row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E25" s="31"/>
+      <x:c r="G25" s="35"/>
+    </x:row>
+    <x:row r="26" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A26" s="12"/>
       <x:c r="B26" s="12"/>
       <x:c r="C26" s="21"/>
       <x:c r="D26" s="32"/>
-      <x:c r="F26" s="35"/>
-    </x:row>
-    <x:row r="27" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E26" s="32"/>
+      <x:c r="G26" s="35"/>
+    </x:row>
+    <x:row r="27" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A27" s="12"/>
       <x:c r="B27" s="12"/>
       <x:c r="C27" s="21"/>
       <x:c r="D27" s="32"/>
-      <x:c r="F27" s="35"/>
-    </x:row>
-    <x:row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E27" s="32"/>
+      <x:c r="G27" s="35"/>
+    </x:row>
+    <x:row r="28" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A28" s="12"/>
       <x:c r="B28" s="12"/>
       <x:c r="C28" s="21"/>
       <x:c r="D28" s="32"/>
-      <x:c r="F28" s="35"/>
-    </x:row>
-    <x:row r="29" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E28" s="32"/>
+      <x:c r="G28" s="35"/>
+    </x:row>
+    <x:row r="29" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A29" s="12"/>
       <x:c r="B29" s="12"/>
       <x:c r="C29" s="21"/>
       <x:c r="D29" s="32"/>
-    </x:row>
-    <x:row r="30" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E29" s="32"/>
+    </x:row>
+    <x:row r="30" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A30" s="12"/>
       <x:c r="B30" s="12"/>
       <x:c r="C30" s="21"/>
       <x:c r="D30" s="32"/>
-    </x:row>
-    <x:row r="31" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E30" s="32"/>
+    </x:row>
+    <x:row r="31" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A31" s="12"/>
       <x:c r="B31" s="12"/>
       <x:c r="C31" s="21"/>
       <x:c r="D31" s="32"/>
-    </x:row>
-    <x:row r="32" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E31" s="32"/>
+    </x:row>
+    <x:row r="32" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A32" s="13"/>
       <x:c r="B32" s="13"/>
       <x:c r="C32" s="22"/>
       <x:c r="D32" s="33"/>
-    </x:row>
-    <x:row r="33" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E32" s="33"/>
+    </x:row>
+    <x:row r="33" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A33" s="13"/>
       <x:c r="B33" s="13"/>
       <x:c r="C33" s="22"/>
       <x:c r="D33" s="33"/>
-    </x:row>
-    <x:row r="34" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E33" s="33"/>
+    </x:row>
+    <x:row r="34" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A34" s="13"/>
       <x:c r="B34" s="13"/>
       <x:c r="C34" s="22"/>
       <x:c r="D34" s="33"/>
-    </x:row>
-    <x:row r="35" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E34" s="33"/>
+    </x:row>
+    <x:row r="35" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A35" s="13"/>
       <x:c r="B35" s="13"/>
       <x:c r="C35" s="22"/>
       <x:c r="D35" s="33"/>
+      <x:c r="E35" s="33"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[Add - Skill Data] GradeDataId 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -19,117 +19,129 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <x:si>
     <x:t>Icon 경로</x:t>
   </x:si>
   <x:si>
+    <x:t>토마토플레어</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>붉은 열기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍의 보호막</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Normal</x:t>
+  </x:si>
+  <x:si>
     <x:t>설명</x:t>
   </x:si>
   <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_RedHeat_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredLevel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_CrimsonShield</x:t>
+  </x:si>
+  <x:si>
+    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>요구 레벨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GradeDataId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Rare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Epic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>사용 가능 횟수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prefab 경로</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxUseCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_TomatoFlare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_RottenTomato</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_CrimsonShield_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skill_TomatoFlare_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Skill_RedHeat</x:t>
+  </x:si>
+  <x:si>
     <x:t>Skill_RottenTomato_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_TomatoFlare_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_RedHeat</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_CrimsonShield_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skill_RedHeat_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>붉은 열기</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍의 보호막</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토마토플레어</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RottenTomato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_CrimsonShield</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_CrimsonShield_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선홍빛 보호막을 생성해 일정 시간 모든 피해를 막아낸다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>썩은 토마토를 바닥에 던져 적에게 지속 피해를 입힌다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_TomatoFlare_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PrefabPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxUseCount</x:t>
-  </x:si>
-  <x:si>
-    <x:t>하늘에서 화염 토마토를 떨어뜨려 폭발 피해를 준다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Skill_RedHeat_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_TomatoFlare</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몸에 붉은빛의 기운을 둘러 공격력을 증가시킨다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Skill_RottenTomato</x:t>
-  </x:si>
-  <x:si>
-    <x:t>사용 가능 횟수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Prefab 경로</x:t>
-  </x:si>
-  <x:si>
-    <x:t>요구 레벨</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RequiredLevel</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1001,7 +1013,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:Q35"/>
+  <x:dimension ref="A1:R35"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="23" style="2" customWidth="1"/>
@@ -1009,88 +1021,96 @@
     <x:col min="3" max="3" width="54.109375" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="16.22265625" style="23" customWidth="1"/>
     <x:col min="5" max="5" width="18.66796875" style="23" customWidth="1"/>
-    <x:col min="6" max="6" width="27.66796875" style="24" customWidth="1"/>
-    <x:col min="7" max="7" width="30.5703125" style="23" customWidth="1"/>
+    <x:col min="6" max="6" width="27.66796875" style="23" customWidth="1"/>
+    <x:col min="7" max="7" width="27.66796875" style="24" customWidth="1"/>
+    <x:col min="8" max="8" width="30.5703125" style="23" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:7" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C1" s="14" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="s">
+      <x:c r="E1" s="25" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="24" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H1" s="23" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A2" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E2" s="25" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F2" s="25" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G2" s="24" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H2" s="23" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A3" s="4" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D3" s="26" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E3" s="26" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F3" s="26" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C1" s="14" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D1" s="25" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="E1" s="25" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F1" s="24" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G1" s="23" t="s">
-        <x:v>34</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:7" ht="15.75" customHeight="1">
-      <x:c r="A2" s="3" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C2" s="14" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D2" s="25" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="E2" s="25" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F2" s="24" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G2" s="23" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:7" ht="15.75" customHeight="1">
-      <x:c r="A3" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B3" s="4" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C3" s="15" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D3" s="26" t="s">
+      <x:c r="G3" s="34" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H3" s="36" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E3" s="26" t="s">
+    </x:row>
+    <x:row r="4" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A4" s="6" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="F3" s="34" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="G3" s="36" t="s">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A4" s="6" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C4" s="16" t="s">
-        <x:v>31</x:v>
       </x:c>
       <x:c r="D4" s="27">
         <x:v>3</x:v>
@@ -1098,13 +1118,15 @@
       <x:c r="E4" s="27">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" s="35" t="s">
-        <x:v>29</x:v>
+      <x:c r="F4" s="27" t="s">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G4" s="35" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H4" s="5"/>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H4" s="35" t="s">
+        <x:v>39</x:v>
+      </x:c>
       <x:c r="I4" s="5"/>
       <x:c r="J4" s="5"/>
       <x:c r="K4" s="5"/>
@@ -1114,16 +1136,17 @@
       <x:c r="O4" s="5"/>
       <x:c r="P4" s="5"/>
       <x:c r="Q4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>3</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>14</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="16" t="s">
-        <x:v>28</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D5" s="27">
         <x:v>3</x:v>
@@ -1131,13 +1154,15 @@
       <x:c r="E5" s="27">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F5" s="35" t="s">
-        <x:v>21</x:v>
+      <x:c r="F5" s="27" t="s">
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G5" s="35" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="H5" s="5"/>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H5" s="35" t="s">
+        <x:v>34</x:v>
+      </x:c>
       <x:c r="I5" s="5"/>
       <x:c r="J5" s="5"/>
       <x:c r="K5" s="5"/>
@@ -1147,16 +1172,17 @@
       <x:c r="O5" s="5"/>
       <x:c r="P5" s="5"/>
       <x:c r="Q5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>9</x:v>
-      </x:c>
       <x:c r="C6" s="17" t="s">
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D6" s="28">
         <x:v>5</x:v>
@@ -1164,13 +1190,15 @@
       <x:c r="E6" s="28">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F6" s="35" t="s">
-        <x:v>16</x:v>
+      <x:c r="F6" s="28" t="s">
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G6" s="35" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="H6" s="5"/>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H6" s="35" t="s">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="I6" s="5"/>
       <x:c r="J6" s="5"/>
       <x:c r="K6" s="5"/>
@@ -1180,16 +1208,17 @@
       <x:c r="O6" s="5"/>
       <x:c r="P6" s="5"/>
       <x:c r="Q6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A7" s="7" t="s">
-        <x:v>5</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>19</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D7" s="28">
         <x:v>4</x:v>
@@ -1197,13 +1226,15 @@
       <x:c r="E7" s="28">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F7" s="35" t="s">
-        <x:v>18</x:v>
+      <x:c r="F7" s="27" t="s">
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G7" s="35" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H7" s="35" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>
@@ -1213,16 +1244,17 @@
       <x:c r="O7" s="5"/>
       <x:c r="P7" s="5"/>
       <x:c r="Q7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A8" s="6"/>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="17"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
-      <x:c r="F8" s="35"/>
+      <x:c r="F8" s="28"/>
       <x:c r="G8" s="35"/>
-      <x:c r="H8" s="5"/>
+      <x:c r="H8" s="35"/>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>
       <x:c r="K8" s="5"/>
@@ -1232,16 +1264,17 @@
       <x:c r="O8" s="5"/>
       <x:c r="P8" s="5"/>
       <x:c r="Q8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A9" s="7"/>
       <x:c r="B9" s="7"/>
       <x:c r="C9" s="17"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
-      <x:c r="F9" s="35"/>
+      <x:c r="F9" s="28"/>
       <x:c r="G9" s="35"/>
-      <x:c r="H9" s="5"/>
+      <x:c r="H9" s="35"/>
       <x:c r="I9" s="5"/>
       <x:c r="J9" s="5"/>
       <x:c r="K9" s="5"/>
@@ -1251,16 +1284,17 @@
       <x:c r="O9" s="5"/>
       <x:c r="P9" s="5"/>
       <x:c r="Q9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A10" s="6"/>
       <x:c r="B10" s="6"/>
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="27"/>
       <x:c r="E10" s="27"/>
-      <x:c r="F10" s="35"/>
+      <x:c r="F10" s="27"/>
       <x:c r="G10" s="35"/>
-      <x:c r="H10" s="5"/>
+      <x:c r="H10" s="35"/>
       <x:c r="I10" s="5"/>
       <x:c r="J10" s="5"/>
       <x:c r="K10" s="5"/>
@@ -1270,16 +1304,17 @@
       <x:c r="O10" s="5"/>
       <x:c r="P10" s="5"/>
       <x:c r="Q10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A11" s="9"/>
       <x:c r="B11" s="9"/>
       <x:c r="C11" s="18"/>
       <x:c r="D11" s="29"/>
       <x:c r="E11" s="29"/>
-      <x:c r="F11" s="35"/>
+      <x:c r="F11" s="29"/>
       <x:c r="G11" s="35"/>
-      <x:c r="H11" s="5"/>
+      <x:c r="H11" s="35"/>
       <x:c r="I11" s="5"/>
       <x:c r="J11" s="5"/>
       <x:c r="K11" s="5"/>
@@ -1289,16 +1324,17 @@
       <x:c r="O11" s="5"/>
       <x:c r="P11" s="5"/>
       <x:c r="Q11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A12" s="8"/>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
-      <x:c r="F12" s="35"/>
+      <x:c r="F12" s="30"/>
       <x:c r="G12" s="35"/>
-      <x:c r="H12" s="5"/>
+      <x:c r="H12" s="35"/>
       <x:c r="I12" s="5"/>
       <x:c r="J12" s="5"/>
       <x:c r="K12" s="5"/>
@@ -1308,16 +1344,17 @@
       <x:c r="O12" s="5"/>
       <x:c r="P12" s="5"/>
       <x:c r="Q12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A13" s="6"/>
       <x:c r="B13" s="6"/>
       <x:c r="C13" s="16"/>
       <x:c r="D13" s="27"/>
       <x:c r="E13" s="27"/>
-      <x:c r="F13" s="35"/>
+      <x:c r="F13" s="27"/>
       <x:c r="G13" s="35"/>
-      <x:c r="H13" s="5"/>
+      <x:c r="H13" s="35"/>
       <x:c r="I13" s="5"/>
       <x:c r="J13" s="5"/>
       <x:c r="K13" s="5"/>
@@ -1327,16 +1364,17 @@
       <x:c r="O13" s="5"/>
       <x:c r="P13" s="5"/>
       <x:c r="Q13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A14" s="9"/>
       <x:c r="B14" s="9"/>
       <x:c r="C14" s="18"/>
       <x:c r="D14" s="29"/>
       <x:c r="E14" s="29"/>
-      <x:c r="F14" s="35"/>
+      <x:c r="F14" s="29"/>
       <x:c r="G14" s="35"/>
-      <x:c r="H14" s="5"/>
+      <x:c r="H14" s="35"/>
       <x:c r="I14" s="5"/>
       <x:c r="J14" s="5"/>
       <x:c r="K14" s="5"/>
@@ -1346,16 +1384,17 @@
       <x:c r="O14" s="5"/>
       <x:c r="P14" s="5"/>
       <x:c r="Q14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A15" s="9"/>
       <x:c r="B15" s="9"/>
       <x:c r="C15" s="18"/>
       <x:c r="D15" s="29"/>
       <x:c r="E15" s="29"/>
-      <x:c r="F15" s="35"/>
+      <x:c r="F15" s="29"/>
       <x:c r="G15" s="35"/>
-      <x:c r="H15" s="5"/>
+      <x:c r="H15" s="35"/>
       <x:c r="I15" s="5"/>
       <x:c r="J15" s="5"/>
       <x:c r="K15" s="5"/>
@@ -1365,152 +1404,173 @@
       <x:c r="O15" s="5"/>
       <x:c r="P15" s="5"/>
       <x:c r="Q15" s="5"/>
-    </x:row>
-    <x:row r="16" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="R15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A16" s="10"/>
       <x:c r="B16" s="10"/>
       <x:c r="C16" s="20"/>
       <x:c r="D16" s="31"/>
       <x:c r="E16" s="31"/>
-    </x:row>
-    <x:row r="17" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F16" s="31"/>
+    </x:row>
+    <x:row r="17" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A17" s="11"/>
       <x:c r="B17" s="11"/>
       <x:c r="C17" s="20"/>
       <x:c r="D17" s="31"/>
       <x:c r="E17" s="31"/>
-    </x:row>
-    <x:row r="18" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F17" s="31"/>
+    </x:row>
+    <x:row r="18" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A18" s="11"/>
       <x:c r="B18" s="11"/>
       <x:c r="C18" s="20"/>
       <x:c r="D18" s="31"/>
       <x:c r="E18" s="31"/>
-    </x:row>
-    <x:row r="19" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F18" s="31"/>
+    </x:row>
+    <x:row r="19" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A19" s="11"/>
       <x:c r="B19" s="11"/>
       <x:c r="C19" s="20"/>
       <x:c r="D19" s="31"/>
       <x:c r="E19" s="31"/>
-      <x:c r="F19" s="35"/>
+      <x:c r="F19" s="31"/>
       <x:c r="G19" s="35"/>
-    </x:row>
-    <x:row r="20" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="H19" s="35"/>
+    </x:row>
+    <x:row r="20" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A20" s="11"/>
       <x:c r="B20" s="11"/>
       <x:c r="C20" s="20"/>
       <x:c r="D20" s="31"/>
       <x:c r="E20" s="31"/>
-    </x:row>
-    <x:row r="21" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F20" s="31"/>
+    </x:row>
+    <x:row r="21" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A21" s="11"/>
       <x:c r="B21" s="11"/>
       <x:c r="C21" s="20"/>
       <x:c r="D21" s="31"/>
       <x:c r="E21" s="31"/>
-    </x:row>
-    <x:row r="22" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F21" s="31"/>
+    </x:row>
+    <x:row r="22" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A22" s="11"/>
       <x:c r="B22" s="11"/>
       <x:c r="C22" s="20"/>
       <x:c r="D22" s="31"/>
       <x:c r="E22" s="31"/>
-    </x:row>
-    <x:row r="23" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F22" s="31"/>
+    </x:row>
+    <x:row r="23" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A23" s="11"/>
       <x:c r="B23" s="11"/>
       <x:c r="C23" s="20"/>
       <x:c r="D23" s="31"/>
       <x:c r="E23" s="31"/>
-    </x:row>
-    <x:row r="24" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F23" s="31"/>
+    </x:row>
+    <x:row r="24" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A24" s="11"/>
       <x:c r="B24" s="11"/>
       <x:c r="C24" s="20"/>
       <x:c r="D24" s="31"/>
       <x:c r="E24" s="31"/>
-    </x:row>
-    <x:row r="25" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F24" s="31"/>
+    </x:row>
+    <x:row r="25" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A25" s="11"/>
       <x:c r="B25" s="11"/>
       <x:c r="C25" s="20"/>
       <x:c r="D25" s="31"/>
       <x:c r="E25" s="31"/>
-      <x:c r="G25" s="35"/>
-    </x:row>
-    <x:row r="26" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F25" s="31"/>
+      <x:c r="H25" s="35"/>
+    </x:row>
+    <x:row r="26" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A26" s="12"/>
       <x:c r="B26" s="12"/>
       <x:c r="C26" s="21"/>
       <x:c r="D26" s="32"/>
       <x:c r="E26" s="32"/>
-      <x:c r="G26" s="35"/>
-    </x:row>
-    <x:row r="27" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F26" s="32"/>
+      <x:c r="H26" s="35"/>
+    </x:row>
+    <x:row r="27" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A27" s="12"/>
       <x:c r="B27" s="12"/>
       <x:c r="C27" s="21"/>
       <x:c r="D27" s="32"/>
       <x:c r="E27" s="32"/>
-      <x:c r="G27" s="35"/>
-    </x:row>
-    <x:row r="28" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F27" s="32"/>
+      <x:c r="H27" s="35"/>
+    </x:row>
+    <x:row r="28" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A28" s="12"/>
       <x:c r="B28" s="12"/>
       <x:c r="C28" s="21"/>
       <x:c r="D28" s="32"/>
       <x:c r="E28" s="32"/>
-      <x:c r="G28" s="35"/>
-    </x:row>
-    <x:row r="29" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F28" s="32"/>
+      <x:c r="H28" s="35"/>
+    </x:row>
+    <x:row r="29" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A29" s="12"/>
       <x:c r="B29" s="12"/>
       <x:c r="C29" s="21"/>
       <x:c r="D29" s="32"/>
       <x:c r="E29" s="32"/>
-    </x:row>
-    <x:row r="30" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F29" s="32"/>
+    </x:row>
+    <x:row r="30" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A30" s="12"/>
       <x:c r="B30" s="12"/>
       <x:c r="C30" s="21"/>
       <x:c r="D30" s="32"/>
       <x:c r="E30" s="32"/>
-    </x:row>
-    <x:row r="31" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F30" s="32"/>
+    </x:row>
+    <x:row r="31" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A31" s="12"/>
       <x:c r="B31" s="12"/>
       <x:c r="C31" s="21"/>
       <x:c r="D31" s="32"/>
       <x:c r="E31" s="32"/>
-    </x:row>
-    <x:row r="32" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F31" s="32"/>
+    </x:row>
+    <x:row r="32" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A32" s="13"/>
       <x:c r="B32" s="13"/>
       <x:c r="C32" s="22"/>
       <x:c r="D32" s="33"/>
       <x:c r="E32" s="33"/>
-    </x:row>
-    <x:row r="33" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F32" s="33"/>
+    </x:row>
+    <x:row r="33" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A33" s="13"/>
       <x:c r="B33" s="13"/>
       <x:c r="C33" s="22"/>
       <x:c r="D33" s="33"/>
       <x:c r="E33" s="33"/>
-    </x:row>
-    <x:row r="34" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F33" s="33"/>
+    </x:row>
+    <x:row r="34" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A34" s="13"/>
       <x:c r="B34" s="13"/>
       <x:c r="C34" s="22"/>
       <x:c r="D34" s="33"/>
       <x:c r="E34" s="33"/>
-    </x:row>
-    <x:row r="35" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F34" s="33"/>
+    </x:row>
+    <x:row r="35" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A35" s="13"/>
       <x:c r="B35" s="13"/>
       <x:c r="C35" s="22"/>
       <x:c r="D35" s="33"/>
       <x:c r="E35" s="33"/>
+      <x:c r="F35" s="33"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>

</xml_diff>